<commit_message>
added AI insight logic
</commit_message>
<xml_diff>
--- a/Project Overview.xlsx
+++ b/Project Overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Divyesh\IFC\IFC_Prisma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80EC04B-030B-486C-8C81-35224419B39E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42EEAC0B-50DA-406E-BF26-0A56F05B6BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{069BF09D-1EB0-44AE-A074-AC094321DB43}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{069BF09D-1EB0-44AE-A074-AC094321DB43}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -212,9 +212,6 @@
     <t>Last 4 completed calendar quarters (date ranges)</t>
   </si>
   <si>
-    <t>3 random months from the last 12 (month date ranges)</t>
-  </si>
-  <si>
     <t>8 random Mon–Fri weeks from last 12 months (excluding current month)</t>
   </si>
   <si>
@@ -228,6 +225,9 @@
   </si>
   <si>
     <t>Prior calendar year (string, e.g. 2024)</t>
+  </si>
+  <si>
+    <t>5 random months from the last 12 (month date ranges)</t>
   </si>
 </sst>
 </file>
@@ -316,9 +316,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -356,7 +356,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -462,7 +462,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -604,7 +604,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -616,7 +616,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.85546875" customWidth="1"/>
-    <col min="2" max="2" width="81.85546875" customWidth="1"/>
+    <col min="2" max="2" width="79.28515625" customWidth="1"/>
     <col min="3" max="3" width="76.42578125" customWidth="1"/>
     <col min="4" max="4" width="19.85546875" customWidth="1"/>
   </cols>
@@ -841,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="C69" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -871,10 +871,10 @@
         <v>48</v>
       </c>
       <c r="B72" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C72" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -885,7 +885,7 @@
         <v>8</v>
       </c>
       <c r="C73" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -896,7 +896,7 @@
         <v>4</v>
       </c>
       <c r="C74" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -907,7 +907,7 @@
         <v>5</v>
       </c>
       <c r="C75" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -918,7 +918,7 @@
         <v>40</v>
       </c>
       <c r="C76" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added AI insights and fixed searchbar bug
</commit_message>
<xml_diff>
--- a/Project Overview.xlsx
+++ b/Project Overview.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Divyesh\IFC\IFC_Prisma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42EEAC0B-50DA-406E-BF26-0A56F05B6BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3368EAFC-089B-4DED-B9B6-FAA0CF3817C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{069BF09D-1EB0-44AE-A074-AC094321DB43}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{069BF09D-1EB0-44AE-A074-AC094321DB43}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="71">
   <si>
     <t>Approved</t>
   </si>
@@ -155,9 +155,6 @@
     <t>Mail will be sent to respective approver with RACM details and user details.</t>
   </si>
   <si>
-    <t>RACM Decision</t>
-  </si>
-  <si>
     <t>Mail will be sent to user. CC = Coordinator</t>
   </si>
   <si>
@@ -228,6 +225,33 @@
   </si>
   <si>
     <t>5 random months from the last 12 (month date ranges)</t>
+  </si>
+  <si>
+    <t>Format</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Coordinator/Approver Creation</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Reminder Emails for first time submission</t>
+  </si>
+  <si>
+    <t>Mail will be sent to process owner. No CC</t>
+  </si>
+  <si>
+    <t>RACM Decision (Approved/Rejected)</t>
+  </si>
+  <si>
+    <t>Unit Assignment to Coordinator/Approver</t>
+  </si>
+  <si>
+    <t>Mail will be sent to user's ID with Unit name</t>
   </si>
 </sst>
 </file>
@@ -612,11 +636,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7344510A-1B15-4CED-8360-74A45E8617FA}">
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.85546875" customWidth="1"/>
-    <col min="2" max="2" width="79.28515625" customWidth="1"/>
+    <col min="1" max="1" width="44.7109375" customWidth="1"/>
+    <col min="2" max="2" width="87.42578125" customWidth="1"/>
     <col min="3" max="3" width="76.42578125" customWidth="1"/>
     <col min="4" max="4" width="19.85546875" customWidth="1"/>
   </cols>
@@ -773,6 +797,9 @@
       <c r="A56" s="3" t="s">
         <v>30</v>
       </c>
+      <c r="C56" s="2" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -781,144 +808,198 @@
       <c r="B58" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>34</v>
-      </c>
-      <c r="B59" t="s">
-        <v>35</v>
-      </c>
-    </row>
+      <c r="C58" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="60" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>64</v>
+      </c>
+      <c r="B60" t="s">
+        <v>33</v>
+      </c>
+      <c r="C60" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="26.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:3" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>69</v>
+      </c>
+      <c r="B62" t="s">
+        <v>70</v>
+      </c>
+      <c r="C62" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>34</v>
+      </c>
+      <c r="B64" t="s">
+        <v>35</v>
+      </c>
+      <c r="C64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>36</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B66" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>38</v>
-      </c>
-      <c r="B61" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>40</v>
-      </c>
-      <c r="B62" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>42</v>
-      </c>
-      <c r="B63" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A68" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B68" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>45</v>
-      </c>
-      <c r="B69" s="5">
-        <v>1</v>
-      </c>
-      <c r="C69" t="s">
-        <v>61</v>
+      <c r="C66" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>66</v>
+      </c>
+      <c r="B68" t="s">
+        <v>67</v>
+      </c>
+      <c r="C68" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>46</v>
-      </c>
-      <c r="B70" s="5">
-        <v>2</v>
+        <v>68</v>
+      </c>
+      <c r="B70" t="s">
+        <v>38</v>
       </c>
       <c r="C70" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>47</v>
-      </c>
-      <c r="B71" s="5">
-        <v>4</v>
-      </c>
-      <c r="C71" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>48</v>
-      </c>
-      <c r="B72" s="5">
-        <v>5</v>
+        <v>39</v>
+      </c>
+      <c r="B72" t="s">
+        <v>40</v>
       </c>
       <c r="C72" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>49</v>
-      </c>
-      <c r="B73" s="5">
-        <v>8</v>
-      </c>
-      <c r="C73" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>50</v>
-      </c>
-      <c r="B74" s="5">
-        <v>4</v>
-      </c>
-      <c r="C74" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>41</v>
+      </c>
+      <c r="B75" t="s">
+        <v>42</v>
+      </c>
+      <c r="C75" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A78" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>44</v>
+      </c>
+      <c r="B79" s="5">
+        <v>1</v>
+      </c>
+      <c r="C79" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>45</v>
+      </c>
+      <c r="B80" s="5">
+        <v>2</v>
+      </c>
+      <c r="C80" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>46</v>
+      </c>
+      <c r="B81" s="5">
+        <v>4</v>
+      </c>
+      <c r="C81" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>47</v>
+      </c>
+      <c r="B82" s="5">
+        <v>5</v>
+      </c>
+      <c r="C82" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>48</v>
+      </c>
+      <c r="B83" s="5">
+        <v>8</v>
+      </c>
+      <c r="C83" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>49</v>
+      </c>
+      <c r="B84" s="5">
+        <v>4</v>
+      </c>
+      <c r="C84" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>50</v>
+      </c>
+      <c r="B85" s="5">
+        <v>5</v>
+      </c>
+      <c r="C85" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>51</v>
       </c>
-      <c r="B75" s="5">
-        <v>5</v>
-      </c>
-      <c r="C75" t="s">
+      <c r="B86" s="5">
+        <v>40</v>
+      </c>
+      <c r="C86" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>52</v>
-      </c>
-      <c r="B76" s="5">
-        <v>40</v>
-      </c>
-      <c r="C76" t="s">
-        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>